<commit_message>
save changes on 1120
</commit_message>
<xml_diff>
--- a/docs/source/examples/notebooks/models/Pressure_wip/Ruihe/Get_Random_sets/Warwick_ageing_Case_5_5/Excel/0_Re_0_Warwick_ageing_Case_5_5.xlsx
+++ b/docs/source/examples/notebooks/models/Pressure_wip/Ruihe/Get_Random_sets/Warwick_ageing_Case_5_5/Excel/0_Re_0_Warwick_ageing_Case_5_5.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH2"/>
+  <dimension ref="A1:BJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,7 +496,7 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Negative inner SEI lithium interstitial diffusivity [m2.s-1]</t>
+          <t>Inner SEI lithium interstitial diffusivity [m2.s-1]</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Ratio of lithium moles to SEI moles</t>
+          <t>Negative ratio of lithium moles to SEI moles</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
@@ -626,105 +626,115 @@
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
+          <t>CDend 1C SOH [%]</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
           <t>CDend Neg Porosity Sep side</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>CDend LLI [%]</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>LLI to sei-on-cracks [%]</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>LLI to LiP [%]</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>LLI to SEI [%]</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>CDend LLI due to LAM [%]</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>LAM_to_Crack_NE [%]</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>LAM_to_Crack_PE [%]</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>LAM_to_Dry [%]</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>CDend LAM_ne_tot [%]</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>CDend LAM_pe_tot [%]</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Cap per kAh</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>1C Cap per kAh</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>LLI% per kAh</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>LAM_ne% per kAh</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>LAM_pe% per kAh</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Vol_Elely_Tot_All_final</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Vol_Elely_JR_All_final</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Width_all_final</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Error_AGE</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Error_RPT</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Log</t>
         </is>
@@ -759,7 +769,7 @@
         <v>25</v>
       </c>
       <c r="N2" t="n">
-        <v>2.500000000000012e-22</v>
+        <v>3.870000000000014e-19</v>
       </c>
       <c r="O2" t="n">
         <v>1</v>
@@ -779,7 +789,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>{'open-circuit potential': 'current sigmoid', 'thermal': 'lumped', 'SEI': 'interstitial-diffusion limited', 'SEI film resistance': 'distributed', 'SEI porosity change': 'true', 'lithium plating': 'partially reversible', 'lithium plating porosity change': 'true', 'particle mechanics': ('swelling and cracking', 'swelling only'), 'loss of active material': 'stress-driven', 'calculate discharge energy': 'true'}</t>
+          <t>{'open-circuit potential': 'current sigmoid', 'thermal': 'lumped', 'SEI': 'interstitial-diffusion limited', 'SEI on cracks': 'true', 'SEI film resistance': 'distributed', 'SEI porosity change': 'true', 'lithium plating': 'partially reversible', 'lithium plating porosity change': 'true', 'particle mechanics': ('swelling and cracking', 'swelling only'), 'loss of active material': 'stress-driven', 'calculate discharge energy': 'true'}</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -804,10 +814,10 @@
         <v>4541</v>
       </c>
       <c r="AA2" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC2" t="n">
         <v>600000000</v>
@@ -822,10 +832,10 @@
         <v>13100</v>
       </c>
       <c r="AG2" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="AH2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="AI2" t="n">
         <v>10</v>
@@ -841,76 +851,82 @@
         </is>
       </c>
       <c r="AL2" t="n">
-        <v>0.1314902777796649</v>
+        <v>0.7678879829084856</v>
       </c>
       <c r="AM2" t="n">
-        <v>96.09522987766366</v>
+        <v>92.76773297128227</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.1947425816355444</v>
+        <v>96.43304953190616</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.09262886080089183</v>
+        <v>0.1976102587640345</v>
       </c>
       <c r="AP2" t="n">
-        <v>0</v>
+        <v>3.255068273992578</v>
       </c>
       <c r="AQ2" t="n">
-        <v>0.006612785995052054</v>
+        <v>0.3664177803810514</v>
       </c>
       <c r="AR2" t="n">
-        <v>-0.0003802567482112794</v>
+        <v>0.08953686959292391</v>
       </c>
       <c r="AS2" t="n">
-        <v>0.08639633155405106</v>
+        <v>0.01686405000468499</v>
       </c>
       <c r="AT2" t="n">
-        <v>0.05743584046743466</v>
+        <v>2.782249574013918</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.08657828175847593</v>
+        <v>0.3810675257839113</v>
       </c>
       <c r="AV2" t="n">
-        <v>0</v>
+        <v>0.5621090581752575</v>
       </c>
       <c r="AW2" t="n">
-        <v>0.05743584046743466</v>
+        <v>2.221158591957746</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.08657828175847593</v>
+        <v>2.602226117741657</v>
       </c>
       <c r="AY2" t="n">
-        <v>-3518.356965975555</v>
+        <v>2.783267650133003</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.7044540658443799</v>
+        <v>-581.3891762159876</v>
       </c>
       <c r="BA2" t="n">
-        <v>0.4368067467594717</v>
+        <v>-581.6299795676688</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.6584386558491654</v>
+        <v>4.238988428577228</v>
       </c>
       <c r="BC2" t="n">
-        <v>5.861647197064517</v>
+        <v>3.388809534283052</v>
       </c>
       <c r="BD2" t="n">
-        <v>5.038594571797771</v>
+        <v>3.624575083973809</v>
       </c>
       <c r="BE2" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="BF2" t="inlineStr">
+        <v>4.990995225695941</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>4.990995225695941</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>1.544905694247068</v>
+      </c>
+      <c r="BH2" t="inlineStr">
         <is>
           <t>Empty</t>
         </is>
       </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BI2" t="inlineStr">
         <is>
           <t>Empty</t>
         </is>
       </c>
-      <c r="BH2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>